<commit_message>
Hakediş icmalini teklif toplamı (691.227,6 TL) ile hizala
Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/Elmalik_Villa_Hakedis_Paketi.xlsx
+++ b/metraj/Elmalik_Villa_Hakedis_Paketi.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Sözleşme matrahı (KDV hariç)</t>
+          <t>Sözleşme matrahı (imalat)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -602,7 +602,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>KDV matrahı</t>
+          <t>Teklif genel toplam (Teklif_1_2328)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -614,78 +614,66 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>KDV (%20)</t>
+          <t>KDV (%20 — teklifte ayrılmamış, faturada)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>138,245.52 TL</t>
+          <t>138,245.52 TL (matrah 691,227.60 TL üzerinden)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Genel toplam (KDV dahil)</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>829,473.12 TL</t>
-        </is>
-      </c>
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="3" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Detaylı fiyatlı kalem toplamı</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>389,261.50 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Detaylı fiyatlı kalem toplamı</t>
+          <t>Diğer kalemler (götürü / birim fiyat teklifte ayrılmamış)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>389,261.50 TL</t>
+          <t>186,761.50 TL</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Diğer kalemler (götürü / birim fiyat teklifte ayrılmamış)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>186,761.50 TL</t>
-        </is>
-      </c>
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Dosya içeriği</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>1) İMALAT LİSTESİ — sözleşme kalemleri | 2) HAKEDİŞ DÖNEM — bu dönem ilerleme | 3) FATURA TASLAĞI | 4) İCMAL</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Dosya içeriği</t>
+          <t>Not</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>1) İMALAT LİSTESİ — sözleşme kalemleri | 2) HAKEDİŞ DÖNEM — bu dönem ilerleme | 3) FATURA TASLAĞI | 4) İCMAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Not</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Hakediş; çift imzalı saha tutanağı ve tamamlanan imalat oranına göre düzenlenir. Götürü kalemlerde yüzde ilerleme kullanılabilir.</t>
         </is>

</xml_diff>